<commit_message>
inclusion of both 1PL and 3PL for final reporting
Added code to include both item and student estimates for comparison
</commit_message>
<xml_diff>
--- a/observed_score_statistics.xlsx
+++ b/observed_score_statistics.xlsx
@@ -672,19 +672,19 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>17.88157894736842</v>
+        <v>19.06578947368421</v>
       </c>
       <c r="C10" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D10" t="n">
-        <v>3.748660579507149</v>
+        <v>4.034304653231795</v>
       </c>
       <c r="E10" t="n">
-        <v>-1.077875653693573</v>
+        <v>-1.082790653621701</v>
       </c>
       <c r="F10" t="n">
-        <v>0.6845333500824702</v>
+        <v>0.6457139671174237</v>
       </c>
       <c r="G10" t="n">
         <v>25</v>

</xml_diff>